<commit_message>
Platine: günstigere JLC-Teile, Option ESP32-S3-WROOM-1U mit externer Antenne
- Flash ZD35Q1GC-IB, Kondensatoren/Dioden/Widerstände auf Basic-Teile und 0402, Layout angepasst
- WROOM-1U auf demselben Footprint: eigene JLCPCB-BOM/CPL (Modulmitte 3,15 mm versetzt),
  Mouser-Option mit Pigtail RP-SMA/U.FL und Knick-Stabantenne, 3D-Modell des 1U
- Gerber, BOM, CPL, Renders und Bestelllisten neu erzeugt

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkZzubjLKyW9odUwvmxTog
</commit_message>
<xml_diff>
--- a/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
+++ b/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
@@ -413,17 +413,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="40" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
-  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
@@ -520,7 +511,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ersatz für GD5F1GQ5UEYIGR (gleiches Gehäuse und Pinbelegung, von spi_nand_flash unterstützt)</t>
+          <t>Ersatz für ZD35Q1GC-IB (gleiches Gehäuse und Pinbelegung, von spi_nand_flash unterstützt)</t>
         </is>
       </c>
     </row>
@@ -709,12 +700,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>MBR140SFT1G</t>
+          <t>1N5819HW-7-F</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>onsemi</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -727,7 +718,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Schottky 40 V 1 A SOD-123FL</t>
+          <t>Schottky 40 V 1 A SOD-123</t>
         </is>
       </c>
       <c r="F10" t="n">
@@ -735,7 +726,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ersatz für SS14 SOD-123FL</t>
+          <t>Ersatz für B5819W</t>
         </is>
       </c>
     </row>
@@ -795,7 +786,11 @@
       <c r="F12" t="n">
         <v>1</v>
       </c>
-      <c r="G12" t="inlineStr"/>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Ersatz für 1N5819WS (als STAT-Diode gleichwertig)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -833,20 +828,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CC1210MKX5R6BB107</t>
+          <t>CL32A107MPVNNNE</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C1,C10</t>
+          <t>C1,C7,C10</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -855,14 +850,14 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CL32A107MQVNNNE</t>
+          <t>CL21A106KAYNNNE</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -871,205 +866,205 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>11</v>
+        <v>33</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C2,C18,C22</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MLCC 100 µF 6,3 V X5R 1210</t>
+          <t>MLCC 10 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CL21A106KAYNNNE</t>
+          <t>GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C2,C18,C22</t>
+          <t>C19,C20</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 25 V X5R 0805</t>
+          <t>MLCC 22 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>GRM21BR61E226ME44L</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>22</v>
+        <v>40</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C19,C20</t>
+          <t>C4,C5,C16</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 25 V X5R 0805</t>
+          <t>MLCC 1 µF 50 V X5R 0603</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CL10A105KB8NNNC</t>
+          <t>CC0603KRX7R9BB104</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>40</v>
+        <v>90</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C4,C5,C16</t>
+          <t>C6,C8,C9,C17,C21,C23,C25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MLCC 1 µF 50 V X5R 0603</t>
+          <t>MLCC 100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CC0603KRX7R9BB104</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C6,C8,C9,C17,C21,C23,C25</t>
+          <t>C26,C27</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 50 V X7R 0603</t>
+          <t>MLCC 100 nF 16 V X7R 0402</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>TAJA106K016RNJ</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera AVX</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C26,C27</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 16 V X7R 0402</t>
+          <t>Tantal 10 µF 16 V Case A</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
-      </c>
-      <c r="G20" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TAJB106K016RNJ</t>
+          <t>RC0603FR-072KL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Kyocera AVX</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tantal 10 µF 16 V Case B</t>
+          <t>2 kΩ 0603</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
-      </c>
+      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RC0603FR-072KL</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1078,27 +1073,27 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R2,R9,R10,R21,R25,R27</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2 kΩ 0603</t>
+          <t>10 kΩ 0603</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1107,27 +1102,27 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>80</v>
+        <v>50</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>R2,R9,R10,R21,R25,R27</t>
+          <t>R3,R4,R6,R12</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>10 kΩ 0603</t>
+          <t>100 kΩ 0603</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-07100RL</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1136,27 +1131,27 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>R3,R4,R6,R12</t>
+          <t>R5,R11</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>100 kΩ 0603</t>
+          <t>100 Ω 0603</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RC0603FR-07100RL</t>
+          <t>RC0603FR-07330RL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1165,27 +1160,27 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>R5,R11</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>100 Ω 0603</t>
+          <t>330 Ω 0603</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RC0603FR-07330RL</t>
+          <t>RC0603FR-075K1L</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1194,27 +1189,27 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R22,R23</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>330 Ω 0603</t>
+          <t>5,1 kΩ 0603</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RC0603FR-075K1L</t>
+          <t>RC0603FR-0775KL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1223,27 +1218,27 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>R22,R23</t>
+          <t>R24</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>5,1 kΩ 0603</t>
+          <t>75 kΩ 0603</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RC0603FR-0775KL</t>
+          <t>RC1206FR-0710RL</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1256,12 +1251,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>75 kΩ 0603</t>
+          <t>10 Ω 1206</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1272,7 +1267,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RC1206FR-0710RL</t>
+          <t>RC0402FR-07100RL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1281,27 +1276,27 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R28,R30,R31,R32,R33,R34</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>10 Ω 1206</t>
+          <t>100 Ω 0402</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RC0402FR-07100RL</t>
+          <t>RC0402FR-071KL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1310,27 +1305,27 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>R28,R30,R31,R32,R33,R34</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>100 Ω 0402</t>
+          <t>1 kΩ 0402</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RC0402FR-071KL</t>
+          <t>RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1343,12 +1338,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1 kΩ 0402</t>
+          <t>10 kΩ 0402</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1359,12 +1354,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RC0402FR-0710KL</t>
+          <t>B3U-1000P</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1372,52 +1367,52 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>SW3,SW4</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>10 kΩ 0402</t>
+          <t>Taster RESET/BOOT</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>B3U-1000P</t>
+          <t>SM07B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>SW3,SW4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Taster RESET/BOOT</t>
+          <t>JST-SH 7-polig liegend</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SM07B-SRSS-TB(LF)(SN)</t>
+          <t>SM04B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1426,27 +1421,27 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J4,J5</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>JST-SH 7-polig liegend</t>
+          <t>JST-SH 4-polig liegend</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN)</t>
+          <t>SM03B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1455,27 +1450,27 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>J4,J5</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>JST-SH 4-polig liegend</t>
+          <t>JST-SH 3-polig liegend</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SM03B-SRSS-TB(LF)(SN)</t>
+          <t>SM02B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1484,27 +1479,27 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>LED1,M1,SW1,SW2</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JST-SH 3-polig liegend</t>
+          <t>JST-SH 2-polig liegend</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SM02B-SRSS-TB(LF)(SN)</t>
+          <t>S2B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1513,27 +1508,27 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>LED1,M1,SW1,SW2</t>
+          <t>BT1,SP1</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>JST-SH 2-polig liegend</t>
+          <t>JST-PH 2-polig liegend</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>S3B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1542,74 +1537,74 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BT1,SP1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>JST-PH 2-polig liegend</t>
+          <t>JST-PH 3-polig liegend</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S3B-PH-SM4-TB(LF)(SN)</t>
+          <t>TSOP34838</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>TSOP 1-6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>JST-PH 3-polig liegend</t>
+          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TSOP34838</t>
+          <t>MFR-25FBF52-100R</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>TSOP 1-6</t>
+          <t>Filter TSOP (R)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
+          <t>100 Ω THT am Sensor</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1620,12 +1615,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-100R</t>
+          <t>EEU-FR1H4R7</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1633,61 +1628,61 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Filter TSOP (R)</t>
+          <t>Filter TSOP (C)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>100 Ω THT am Sensor</t>
+          <t>Elko 4,7 µF 50 V radial am Sensor</t>
         </is>
       </c>
       <c r="F41" t="n">
         <v>6</v>
       </c>
-      <c r="G41" t="inlineStr"/>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>EEU-FR1H4R7</t>
+          <t>TSAL6100</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Filter TSOP (C)</t>
+          <t>IR-LED</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Elko 4,7 µF 50 V radial am Sensor</t>
+          <t>IR-LED 940 nm 5 mm</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>6</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TSAL6100</t>
+          <t>D2F-01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1695,12 +1690,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>IR-LED</t>
+          <t>Abzugsschalter</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>IR-LED 940 nm 5 mm</t>
+          <t>Mikroschalter</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -1711,12 +1706,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>D2F-01</t>
+          <t>PTS645SL50-2 LFS</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1724,28 +1719,32 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Abzugsschalter</t>
+          <t>Nachladetaster</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mikroschalter</t>
+          <t>Taster 6x6x5 THT</t>
         </is>
       </c>
       <c r="F44" t="n">
         <v>1</v>
       </c>
-      <c r="G44" t="inlineStr"/>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Ersatz für K2-1102DP</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PTS645SL50-2 LFS</t>
+          <t>PEC11R-4215F-S0024</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1753,12 +1752,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Nachladetaster</t>
+          <t>Drehgeber</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Taster 6x6x5 THT</t>
+          <t>Drehgeber 24 Rasten mit Taster</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -1766,47 +1765,43 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Ersatz für K2-1102DP</t>
+          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PEC11R-4215F-S0024</t>
+          <t>SHR-02V-S-B</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Drehgeber</t>
+          <t>Gegenstecker SH 2p</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Drehgeber 24 Rasten mit Taster</t>
+          <t>Gehäuse SH 2-polig</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SHR-02V-S-B</t>
+          <t>SHR-03V-S-B</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1815,27 +1810,27 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 2p</t>
+          <t>Gegenstecker SH 3p</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Gehäuse SH 2-polig</t>
+          <t>Gehäuse SH 3-polig</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SHR-03V-S-B</t>
+          <t>SHR-04V-S-B</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1844,27 +1839,27 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 3p</t>
+          <t>Gegenstecker SH 4p</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Gehäuse SH 3-polig</t>
+          <t>Gehäuse SH 4-polig</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SHR-04V-S-B</t>
+          <t>SHR-07V-S-B</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1873,27 +1868,27 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 4p</t>
+          <t>Gegenstecker SH 7p</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Gehäuse SH 4-polig</t>
+          <t>Gehäuse SH 7-polig</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SHR-07V-S-B</t>
+          <t>SSH-003T-P0.2-H</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1902,27 +1897,27 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>286</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 7p</t>
+          <t>Kontakte SH</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Gehäuse SH 7-polig</t>
+          <t>Crimpkontakt SH AWG 32-28</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
       <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>PHR-2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1931,27 +1926,27 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>286</v>
+        <v>20</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Kontakte SH</t>
+          <t>Gegenstecker PH 2p</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Crimpkontakt SH AWG 32-28</t>
+          <t>Gehäuse PH 2-polig</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PHR-2</t>
+          <t>PHR-3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1960,27 +1955,27 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 2p</t>
+          <t>Gegenstecker PH 3p</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Gehäuse PH 2-polig</t>
+          <t>Gehäuse PH 3-polig</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PHR-3</t>
+          <t>SPH-002T-P0.5S</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1989,51 +1984,22 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>10</v>
+        <v>77</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 3p</t>
+          <t>Kontakte PH</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Gehäuse PH 3-polig</t>
+          <t>Crimpkontakt PH AWG 30-24</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="G53" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>SPH-002T-P0.5S</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>JST</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>77</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Kontakte PH</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Crimpkontakt PH AWG 30-24</t>
-        </is>
-      </c>
-      <c r="F54" t="n">
-        <v>7</v>
-      </c>
-      <c r="G54" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Platine: microSD-Slot gedreht, Ein/Aus über den Drehgeber-Taster, R7 12 Ω, 10 µF am Slot
- J7: Karte wird auf der Kontaktseite eingesteckt (Datenblatt TF-018) -> Slot gedreht, Kontakte und
  Öffnung an der Unterkante, SD-Leitungen neu verlegt
- Soft-Power: Q4 (AO3401A) trennt den Akku von BAT_SW, Taster an J5.2 schaltet über D6 (BAT54CW) ein,
  IO21 hält über Q5, IO9 liest den Taster; Lasche oben links 18,6 x 9 mm mit den neuen Teilen,
  Leitungen auf B.Cu über die Oberkante, Akku-Plus über In2
- R7 12 Ω (C17913), C28 10 µF an der microSD-Versorgung
- Gerber, BOM/CPL (alle Varianten), Mouser-BOM, Renders und Doku neu

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkZzubjLKyW9odUwvmxTog
</commit_message>
<xml_diff>
--- a/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
+++ b/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,7 +480,6 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -542,7 +541,6 @@
       <c r="F4" t="n">
         <v>1</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -604,7 +602,6 @@
       <c r="F6" t="n">
         <v>1</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -633,7 +630,6 @@
       <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -662,7 +658,6 @@
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -676,11 +671,11 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Q1,Q2</t>
+          <t>Q1,Q2,Q5</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -689,7 +684,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -700,7 +695,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>1N5819HW-7-F</t>
+          <t>DMP3099L-7</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -709,65 +704,69 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D1,D4</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Schottky 40 V 1 A SOD-123</t>
+          <t>P-MOSFET 30 V SOT-23 (Ein/Aus)</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ersatz für B5819W</t>
+          <t>Ersatz für AO3401A (gleiche Pinbelegung)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SS34-E3/57T</t>
+          <t>1N5819HW-7-F</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D1,D4</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Schottky 40 V 3 A SMA</t>
+          <t>Schottky 40 V 1 A SOD-123</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Ersatz für B5819W</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BAT54WS-7-F</t>
+          <t>SS34-E3/57T</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -775,32 +774,27 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Schottky 30 V SOD-323</t>
+          <t>Schottky 40 V 3 A SMA</t>
         </is>
       </c>
       <c r="F12" t="n">
         <v>1</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>Ersatz für 1N5819WS (als STAT-Diode gleichwertig)</t>
-        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SRP5030T-100M</t>
+          <t>BAT54WS-7-F</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -808,12 +802,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Speicherdrossel 10 µH 5,7x5,2</t>
+          <t>Schottky 30 V SOD-323</t>
         </is>
       </c>
       <c r="F13" t="n">
@@ -821,101 +815,103 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Ersatz für Sunlord MWSA0503S-100MT (Pads überlappen)</t>
+          <t>Ersatz für 1N5819WS (als STAT-Diode gleichwertig)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CL32A107MPVNNNE</t>
+          <t>BAT54CW-7-F</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C1,C7,C10</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MLCC 100 µF 10 V X5R 1210</t>
+          <t>Doppel-Schottky gemeinsame Kathode SOT-323 (Ein/Aus-Taster)</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
-      </c>
-      <c r="G14" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CL21A106KAYNNNE</t>
+          <t>SRP5030T-100M</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>33</v>
+        <v>10</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C2,C18,C22</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 25 V X5R 0805</t>
+          <t>Speicherdrossel 10 µH 5,7x5,2</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
-      </c>
-      <c r="G15" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Ersatz für Sunlord MWSA0503S-100MT (Pads überlappen)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GRM21BR61E226ME44L</t>
+          <t>CL32A107MPVNNNE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C19,C20</t>
+          <t>C1,C7,C10</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 25 V X5R 0805</t>
+          <t>MLCC 100 µF 10 V X5R 1210</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" t="inlineStr"/>
+        <v>3</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CL10A105KB8NNNC</t>
+          <t>CL21A106KAYNNNE</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -924,118 +920,110 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C4,C5,C16</t>
+          <t>C2,C18,C22</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MLCC 1 µF 50 V X5R 0603</t>
+          <t>MLCC 10 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>3</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CC0603KRX7R9BB104</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>90</v>
+        <v>20</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C6,C8,C9,C17,C21,C23,C25</t>
+          <t>C28</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 50 V X7R 0603</t>
+          <t>MLCC 10 µF 10 V X5R 0603 (microSD)</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>7</v>
-      </c>
-      <c r="G18" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C26,C27</t>
+          <t>C19,C20</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 16 V X7R 0402</t>
+          <t>MLCC 22 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F19" t="n">
         <v>2</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TAJA106K016RNJ</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kyocera AVX</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C4,C5,C16</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tantal 10 µF 16 V Case A</t>
+          <t>MLCC 1 µF 50 V X5R 0603</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RC0603FR-072KL</t>
+          <t>CC0603KRX7R9BB104</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1044,85 +1032,87 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>C6,C8,C9,C17,C21,C23,C25</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>2 kΩ 0603</t>
+          <t>MLCC 100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" t="inlineStr"/>
+        <v>7</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>R2,R9,R10,R21,R25,R27</t>
+          <t>C26,C27</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>10 kΩ 0603</t>
+          <t>MLCC 100 nF 16 V X7R 0402</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>6</v>
-      </c>
-      <c r="G22" t="inlineStr"/>
+        <v>2</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>TAJA106K016RNJ</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Kyocera AVX</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>R3,R4,R6,R12</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>100 kΩ 0603</t>
+          <t>Tantal 10 µF 16 V Case A</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
-      </c>
-      <c r="G23" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RC0603FR-07100RL</t>
+          <t>RC0603FR-072KL</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1131,27 +1121,26 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>R5,R11</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>100 Ω 0603</t>
+          <t>2 kΩ 0603</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
-      </c>
-      <c r="G24" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RC0603FR-07330RL</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1160,27 +1149,26 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R2,R9,R10,R21,R25,R27</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>330 Ω 0603</t>
+          <t>10 kΩ 0603</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
-      </c>
-      <c r="G25" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RC0603FR-075K1L</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1189,27 +1177,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>30</v>
+        <v>70</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R22,R23</t>
+          <t>R3,R4,R6,R12,R38,R40</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>5,1 kΩ 0603</t>
+          <t>100 kΩ 0603</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
-      </c>
-      <c r="G26" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RC0603FR-0775KL</t>
+          <t>RC0603FR-07100RL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1218,27 +1205,26 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>R5,R11</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>75 kΩ 0603</t>
+          <t>100 Ω 0603</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
-      </c>
-      <c r="G27" t="inlineStr"/>
+        <v>2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RC1206FR-0710RL</t>
+          <t>RC0603FR-07330RL</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1251,23 +1237,22 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>10 Ω 1206</t>
+          <t>330 Ω 0603</t>
         </is>
       </c>
       <c r="F28" t="n">
         <v>1</v>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RC0402FR-07100RL</t>
+          <t>RC0603FR-075K1L</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1276,27 +1261,26 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>R28,R30,R31,R32,R33,R34</t>
+          <t>R22,R23</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>100 Ω 0402</t>
+          <t>5,1 kΩ 0603</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>6</v>
-      </c>
-      <c r="G29" t="inlineStr"/>
+        <v>2</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RC0402FR-071KL</t>
+          <t>RC0603FR-0775KL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1309,23 +1293,22 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R24</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1 kΩ 0402</t>
+          <t>75 kΩ 0603</t>
         </is>
       </c>
       <c r="F30" t="n">
         <v>1</v>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RC0402FR-0710KL</t>
+          <t>RC1206FR-0712RL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1338,86 +1321,83 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>10 kΩ 0402</t>
+          <t>12 Ω 1206</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>B3U-1000P</t>
+          <t>RC0402FR-07100RL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>SW3,SW4</t>
+          <t>R28,R30,R31,R32,R33,R34</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Taster RESET/BOOT</t>
+          <t>100 Ω 0402</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
-      </c>
-      <c r="G32" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SM07B-SRSS-TB(LF)(SN)</t>
+          <t>RC0402FR-071KL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>JST-SH 7-polig liegend</t>
+          <t>1 kΩ 0402</t>
         </is>
       </c>
       <c r="F33" t="n">
         <v>1</v>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN)</t>
+          <t>RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1425,52 +1405,50 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>J4,J5</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>JST-SH 4-polig liegend</t>
+          <t>10 kΩ 0402</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
-      </c>
-      <c r="G34" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SM03B-SRSS-TB(LF)(SN)</t>
+          <t>B3U-1000P</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>SW3,SW4</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>JST-SH 3-polig liegend</t>
+          <t>Taster RESET/BOOT</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" t="inlineStr"/>
+        <v>2</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SM02B-SRSS-TB(LF)(SN)</t>
+          <t>SM07B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1479,27 +1457,26 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LED1,M1,SW1,SW2</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JST-SH 2-polig liegend</t>
+          <t>JST-SH 7-polig liegend</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>4</v>
-      </c>
-      <c r="G36" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>SM04B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1512,23 +1489,22 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>BT1,SP1</t>
+          <t>J4,J5</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>JST-PH 2-polig liegend</t>
+          <t>JST-SH 4-polig liegend</t>
         </is>
       </c>
       <c r="F37" t="n">
         <v>2</v>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>S3B-PH-SM4-TB(LF)(SN)</t>
+          <t>SM03B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1541,114 +1517,106 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>JST-PH 3-polig liegend</t>
+          <t>JST-SH 3-polig liegend</t>
         </is>
       </c>
       <c r="F38" t="n">
         <v>1</v>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TSOP34838</t>
+          <t>SM02B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>TSOP 1-6</t>
+          <t>LED1,M1,SW1,SW2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
+          <t>JST-SH 2-polig liegend</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>6</v>
-      </c>
-      <c r="G39" t="inlineStr"/>
+        <v>4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-100R</t>
+          <t>S2B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Filter TSOP (R)</t>
+          <t>BT1,SP1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>100 Ω THT am Sensor</t>
+          <t>JST-PH 2-polig liegend</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>6</v>
-      </c>
-      <c r="G40" t="inlineStr"/>
+        <v>2</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>EEU-FR1H4R7</t>
+          <t>S3B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Filter TSOP (C)</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Elko 4,7 µF 50 V radial am Sensor</t>
+          <t>JST-PH 3-polig liegend</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>6</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TSAL6100</t>
+          <t>TSOP34838</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1657,94 +1625,92 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>IR-LED</t>
+          <t>TSOP 1-6</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>IR-LED 940 nm 5 mm</t>
+          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>1</v>
-      </c>
-      <c r="G42" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>D2F-01</t>
+          <t>MFR-25FBF52-100R</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Abzugsschalter</t>
+          <t>Filter TSOP (R)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mikroschalter</t>
+          <t>100 Ω THT am Sensor</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" t="inlineStr"/>
+        <v>6</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PTS645SL50-2 LFS</t>
+          <t>EEU-FR1H4R7</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Nachladetaster</t>
+          <t>Filter TSOP (C)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Taster 6x6x5 THT</t>
+          <t>Elko 4,7 µF 50 V radial am Sensor</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Ersatz für K2-1102DP</t>
+          <t>Polung beachten</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PEC11R-4215F-S0024</t>
+          <t>TSAL6100</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1752,61 +1718,55 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Drehgeber</t>
+          <t>IR-LED</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Drehgeber 24 Rasten mit Taster</t>
+          <t>IR-LED 940 nm 5 mm</t>
         </is>
       </c>
       <c r="F45" t="n">
         <v>1</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
-        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SHR-02V-S-B</t>
+          <t>D2F-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 2p</t>
+          <t>Abzugsschalter</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Gehäuse SH 2-polig</t>
+          <t>Mikroschalter</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>4</v>
-      </c>
-      <c r="G46" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SHR-03V-S-B</t>
+          <t>PTS645SL50-2 LFS</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1814,52 +1774,60 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 3p</t>
+          <t>Nachladetaster</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Gehäuse SH 3-polig</t>
+          <t>Taster 6x6x5 THT</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>1</v>
       </c>
-      <c r="G47" t="inlineStr"/>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Ersatz für K2-1102DP</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SHR-04V-S-B</t>
+          <t>PEC11R-4215F-S0024</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 4p</t>
+          <t>Drehgeber</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Gehäuse SH 4-polig</t>
+          <t>Drehgeber 24 Rasten mit Taster</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>2</v>
-      </c>
-      <c r="G48" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SHR-07V-S-B</t>
+          <t>SHR-02V-S-B</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1868,27 +1836,26 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 7p</t>
+          <t>Gegenstecker SH 2p</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Gehäuse SH 7-polig</t>
+          <t>Gehäuse SH 2-polig</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" t="inlineStr"/>
+        <v>4</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>SHR-03V-S-B</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1897,27 +1864,26 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>286</v>
+        <v>10</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Kontakte SH</t>
+          <t>Gegenstecker SH 3p</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Crimpkontakt SH AWG 32-28</t>
+          <t>Gehäuse SH 3-polig</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>26</v>
-      </c>
-      <c r="G50" t="inlineStr"/>
+        <v>1</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>PHR-2</t>
+          <t>SHR-04V-S-B</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1930,23 +1896,22 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 2p</t>
+          <t>Gegenstecker SH 4p</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Gehäuse PH 2-polig</t>
+          <t>Gehäuse SH 4-polig</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>2</v>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PHR-3</t>
+          <t>SHR-07V-S-B</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1959,47 +1924,129 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 3p</t>
+          <t>Gegenstecker SH 7p</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Gehäuse PH 3-polig</t>
+          <t>Gehäuse SH 7-polig</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>1</v>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
+          <t>SSH-003T-P0.2-H</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>286</v>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Kontakte SH</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Crimpkontakt SH AWG 32-28</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>PHR-2</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>20</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Gegenstecker PH 2p</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Gehäuse PH 2-polig</t>
+        </is>
+      </c>
+      <c r="F54" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>PHR-3</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Gegenstecker PH 3p</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Gehäuse PH 3-polig</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
           <t>SPH-002T-P0.5S</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B56" t="inlineStr">
         <is>
           <t>JST</t>
         </is>
       </c>
-      <c r="C53" t="n">
+      <c r="C56" t="n">
         <v>77</v>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D56" t="inlineStr">
         <is>
           <t>Kontakte PH</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E56" t="inlineStr">
         <is>
           <t>Crimpkontakt PH AWG 30-24</t>
         </is>
       </c>
-      <c r="F53" t="n">
+      <c r="F56" t="n">
         <v>7</v>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Platine: IP5306 (2 A Laden + 5 V) statt MT3608/MCP73831, Ein/Aus über KEY, eigener I²C-Bus
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkZzubjLKyW9odUwvmxTog
</commit_message>
<xml_diff>
--- a/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
+++ b/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G56"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -517,12 +517,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>MCP73831T-2ACI/OT</t>
+          <t>LM1117MPX-3.3/NOPB</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Microchip</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -530,27 +530,32 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>U3</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Li-Ion-Lader SOT-23-5</t>
+          <t>LDO 3,3 V SOT-223</t>
         </is>
       </c>
       <c r="F4" t="n">
         <v>1</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Ersatz für AMS1117-3.3 (gleiche Pinbelegung)</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>LM1117MPX-3.3/NOPB</t>
+          <t>74HCT125PW,118</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Texas Instruments</t>
+          <t>Nexperia</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -558,32 +563,27 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>U2</t>
+          <t>U5</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>LDO 3,3 V SOT-223</t>
+          <t>Puffer TSSOP-14</t>
         </is>
       </c>
       <c r="F5" t="n">
         <v>1</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>Ersatz für AMS1117-3.3 (gleiche Pinbelegung)</t>
-        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>74HCT125PW,118</t>
+          <t>MAX98357AETE+T</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>Analog Devices / Maxim</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -591,12 +591,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Puffer TSSOP-14</t>
+          <t>I2S-Verstärker TQFN-16</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -606,12 +606,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MAX98357AETE+T</t>
+          <t>USBLC6-2SC6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Analog Devices / Maxim</t>
+          <t>STMicroelectronics</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -619,12 +619,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>I2S-Verstärker TQFN-16</t>
+          <t>USB-ESD SOT-23-6</t>
         </is>
       </c>
       <c r="F7" t="n">
@@ -634,35 +634,40 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>USBLC6-2SC6</t>
+          <t>DMN3404L-7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>STMicroelectronics</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>Q1,Q2</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>USB-ESD SOT-23-6</t>
+          <t>N-MOSFET 30 V SOT-23</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Ersatz für AO3400A (gleiche Pinbelegung)</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DMN3404L-7</t>
+          <t>1N5819HW-7-F</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -671,31 +676,31 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Q1,Q2,Q5</t>
+          <t>D1,D4</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>N-MOSFET 30 V SOT-23</t>
+          <t>Schottky 40 V 1 A SOD-123</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Ersatz für AO3400A (gleiche Pinbelegung)</t>
+          <t>Ersatz für B5819W</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>DMP3099L-7</t>
+          <t>BAT54CW-7-F</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -708,182 +713,167 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>P-MOSFET 30 V SOT-23 (Ein/Aus)</t>
+          <t>Doppel-Schottky gemeinsame Kathode SOT-323 (Ein/Aus-Taster)</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Ersatz für AO3401A (gleiche Pinbelegung)</t>
-        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>1N5819HW-7-F</t>
+          <t>SRP5030T-1R0M</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>D1,D4</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Schottky 40 V 1 A SOD-123</t>
+          <t>Speicherdrossel 1 µH 5,7x5,2 (IP5306)</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ersatz für B5819W</t>
+          <t>Ersatz für Sunlord MWSA0503S-1R0MT (Pads überlappen)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SS34-E3/57T</t>
+          <t>CL32A107MPVNNNE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>C1,C7,C10</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Schottky 40 V 3 A SMA</t>
+          <t>MLCC 100 µF 10 V X5R 1210</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BAT54WS-7-F</t>
+          <t>CL21A106KAYNNNE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>C2,C4,C18,C22</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Schottky 30 V SOD-323</t>
+          <t>MLCC 10 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Ersatz für 1N5819WS (als STAT-Diode gleichwertig)</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BAT54CW-7-F</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>C28,C29</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Doppel-Schottky gemeinsame Kathode SOT-323 (Ein/Aus-Taster)</t>
+          <t>MLCC 10 µF 10 V X5R 0603</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SRP5030T-100M</t>
+          <t>GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>C19,C20,C30</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Speicherdrossel 10 µH 5,7x5,2</t>
+          <t>MLCC 22 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>Ersatz für Sunlord MWSA0503S-100MT (Pads überlappen)</t>
-        </is>
+        <v>3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CL32A107MPVNNNE</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -892,26 +882,26 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C1,C7,C10</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MLCC 100 µF 10 V X5R 1210</t>
+          <t>MLCC 1 µF 50 V X5R 0603</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CL21A106KAYNNNE</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -920,72 +910,72 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C2,C18,C22</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 25 V X5R 0805</t>
+          <t>MLCC 22 µF 6,3 V X5R 0603 (IP5306 BAT)</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>CC0603KRX7R9BB104</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C28</t>
+          <t>C6,C8,C9,C17,C21,C23,C25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 10 V X5R 0603 (microSD)</t>
+          <t>MLCC 100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>GRM21BR61E226ME44L</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C19,C20</t>
+          <t>C26,C27</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 25 V X5R 0805</t>
+          <t>MLCC 100 nF 16 V X7R 0402</t>
         </is>
       </c>
       <c r="F19" t="n">
@@ -995,35 +985,40 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CL10A105KB8NNNC</t>
+          <t>TAJA106K016RNJ</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera AVX</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>40</v>
+        <v>11</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C4,C5,C16</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>MLCC 1 µF 50 V X5R 0603</t>
+          <t>Tantal 10 µF 16 V Case A</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CC0603KRX7R9BB104</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1032,31 +1027,31 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>C6,C8,C9,C17,C21,C23,C25</t>
+          <t>R9,R10,R21,R24,R27</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 50 V X7R 0603</t>
+          <t>10 kΩ 0603</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1064,12 +1059,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>C26,C27</t>
+          <t>R6,R12</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 16 V X7R 0402</t>
+          <t>100 kΩ 0603</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -1079,40 +1074,35 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TAJA106K016RNJ</t>
+          <t>RC0603FR-071ML</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Kyocera AVX</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>R3,R4</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Tantal 10 µF 16 V Case A</t>
+          <t>1 MΩ 0603</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RC0603FR-072KL</t>
+          <t>RC0603FR-072RL</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1130,7 +1120,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2 kΩ 0603</t>
+          <t>2 Ω 0603</t>
         </is>
       </c>
       <c r="F24" t="n">
@@ -1140,7 +1130,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603FR-071RL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1149,26 +1139,26 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>R2,R9,R10,R21,R25,R27</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>10 kΩ 0603</t>
+          <t>1 Ω 0603</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-07100RL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1177,26 +1167,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R3,R4,R6,R12,R38,R40</t>
+          <t>R5,R11</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>100 kΩ 0603</t>
+          <t>100 Ω 0603</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RC0603FR-07100RL</t>
+          <t>RC0603FR-07330RL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1205,26 +1195,26 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>R5,R11</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>100 Ω 0603</t>
+          <t>330 Ω 0603</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RC0603FR-07330RL</t>
+          <t>RC0603FR-075K1L</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1233,26 +1223,26 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R22,R23</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>330 Ω 0603</t>
+          <t>5,1 kΩ 0603</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RC0603FR-075K1L</t>
+          <t>RC1206FR-0712RL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1261,26 +1251,26 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>R22,R23</t>
+          <t>R7</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>5,1 kΩ 0603</t>
+          <t>12 Ω 1206</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RC0603FR-0775KL</t>
+          <t>RC0402FR-07100RL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1289,26 +1279,26 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>R24</t>
+          <t>R28,R30,R31,R32,R33,R34</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>75 kΩ 0603</t>
+          <t>100 Ω 0402</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RC1206FR-0712RL</t>
+          <t>RC0402FR-071KL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1321,12 +1311,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>12 Ω 1206</t>
+          <t>1 kΩ 0402</t>
         </is>
       </c>
       <c r="F31" t="n">
@@ -1336,7 +1326,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RC0402FR-07100RL</t>
+          <t>RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1345,26 +1335,26 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>R28,R30,R31,R32,R33,R34</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>100 Ω 0402</t>
+          <t>10 kΩ 0402</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RC0402FR-071KL</t>
+          <t>RC0402FR-074K7L</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1373,31 +1363,31 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R38,R40</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1 kΩ 0402</t>
+          <t>4,7 kΩ 0402</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RC0402FR-0710KL</t>
+          <t>B3U-1000P</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1405,50 +1395,50 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>SW3,SW4</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>10 kΩ 0402</t>
+          <t>Taster RESET/BOOT</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>B3U-1000P</t>
+          <t>SM07B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>SW3,SW4</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Taster RESET/BOOT</t>
+          <t>JST-SH 7-polig liegend</t>
         </is>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SM07B-SRSS-TB(LF)(SN)</t>
+          <t>SM04B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1457,26 +1447,26 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>J4,J5</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JST-SH 7-polig liegend</t>
+          <t>JST-SH 4-polig liegend</t>
         </is>
       </c>
       <c r="F36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN)</t>
+          <t>SM03B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1485,26 +1475,26 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>J4,J5</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>JST-SH 4-polig liegend</t>
+          <t>JST-SH 3-polig liegend</t>
         </is>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SM03B-SRSS-TB(LF)(SN)</t>
+          <t>SM02B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1513,26 +1503,26 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>LED1,M1,SW1,SW2</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>JST-SH 3-polig liegend</t>
+          <t>JST-SH 2-polig liegend</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SM02B-SRSS-TB(LF)(SN)</t>
+          <t>S2B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1541,26 +1531,26 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>LED1,M1,SW1,SW2</t>
+          <t>BT1,SP1</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>JST-SH 2-polig liegend</t>
+          <t>JST-PH 2-polig liegend</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>S3B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1569,72 +1559,72 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>BT1,SP1</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>JST-PH 2-polig liegend</t>
+          <t>JST-PH 3-polig liegend</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>S3B-PH-SM4-TB(LF)(SN)</t>
+          <t>TSOP34838</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>TSOP 1-6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>JST-PH 3-polig liegend</t>
+          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TSOP34838</t>
+          <t>MFR-25FBF52-100R</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>TSOP 1-6</t>
+          <t>Filter TSOP (R)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
+          <t>100 Ω THT am Sensor</t>
         </is>
       </c>
       <c r="F42" t="n">
@@ -1644,12 +1634,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-100R</t>
+          <t>EEU-FR1H4R7</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1657,60 +1647,60 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Filter TSOP (R)</t>
+          <t>Filter TSOP (C)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>100 Ω THT am Sensor</t>
+          <t>Elko 4,7 µF 50 V radial am Sensor</t>
         </is>
       </c>
       <c r="F43" t="n">
         <v>6</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>EEU-FR1H4R7</t>
+          <t>TSAL6100</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Filter TSOP (C)</t>
+          <t>IR-LED</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Elko 4,7 µF 50 V radial am Sensor</t>
+          <t>IR-LED 940 nm 5 mm</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>6</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TSAL6100</t>
+          <t>D2F-01</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1718,12 +1708,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>IR-LED</t>
+          <t>Abzugsschalter</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>IR-LED 940 nm 5 mm</t>
+          <t>Mikroschalter</t>
         </is>
       </c>
       <c r="F45" t="n">
@@ -1733,12 +1723,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>D2F-01</t>
+          <t>PTS645SL50-2 LFS</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1746,27 +1736,32 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Abzugsschalter</t>
+          <t>Nachladetaster</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Mikroschalter</t>
+          <t>Taster 6x6x5 THT</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>1</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Ersatz für K2-1102DP</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PTS645SL50-2 LFS</t>
+          <t>PEC11R-4215F-S0024</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1774,12 +1769,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Nachladetaster</t>
+          <t>Drehgeber</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Taster 6x6x5 THT</t>
+          <t>Drehgeber 24 Rasten mit Taster</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -1787,47 +1782,42 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Ersatz für K2-1102DP</t>
+          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PEC11R-4215F-S0024</t>
+          <t>SHR-02V-S-B</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Drehgeber</t>
+          <t>Gegenstecker SH 2p</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Drehgeber 24 Rasten mit Taster</t>
+          <t>Gehäuse SH 2-polig</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
-        </is>
+        <v>4</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SHR-02V-S-B</t>
+          <t>SHR-03V-S-B</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1836,26 +1826,26 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 2p</t>
+          <t>Gegenstecker SH 3p</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Gehäuse SH 2-polig</t>
+          <t>Gehäuse SH 3-polig</t>
         </is>
       </c>
       <c r="F49" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SHR-03V-S-B</t>
+          <t>SHR-04V-S-B</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1864,26 +1854,26 @@
         </is>
       </c>
       <c r="C50" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 3p</t>
+          <t>Gegenstecker SH 4p</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Gehäuse SH 3-polig</t>
+          <t>Gehäuse SH 4-polig</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SHR-04V-S-B</t>
+          <t>SHR-07V-S-B</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1892,26 +1882,26 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 4p</t>
+          <t>Gegenstecker SH 7p</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Gehäuse SH 4-polig</t>
+          <t>Gehäuse SH 7-polig</t>
         </is>
       </c>
       <c r="F51" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SHR-07V-S-B</t>
+          <t>SSH-003T-P0.2-H</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1920,26 +1910,26 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>10</v>
+        <v>286</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 7p</t>
+          <t>Kontakte SH</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Gehäuse SH 7-polig</t>
+          <t>Crimpkontakt SH AWG 32-28</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>PHR-2</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1948,26 +1938,26 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>286</v>
+        <v>20</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Kontakte SH</t>
+          <t>Gegenstecker PH 2p</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Crimpkontakt SH AWG 32-28</t>
+          <t>Gehäuse PH 2-polig</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>26</v>
+        <v>2</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PHR-2</t>
+          <t>PHR-3</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1976,26 +1966,26 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 2p</t>
+          <t>Gegenstecker PH 3p</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Gehäuse PH 2-polig</t>
+          <t>Gehäuse PH 3-polig</t>
         </is>
       </c>
       <c r="F54" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PHR-3</t>
+          <t>SPH-002T-P0.5S</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2004,47 +1994,19 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>10</v>
+        <v>77</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 3p</t>
+          <t>Kontakte PH</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Gehäuse PH 3-polig</t>
+          <t>Crimpkontakt PH AWG 30-24</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>SPH-002T-P0.5S</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>JST</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>77</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Kontakte PH</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Crimpkontakt PH AWG 30-24</t>
-        </is>
-      </c>
-      <c r="F56" t="n">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Platine: Stecker zusammengelegt, Basic-Teile, MOSFET-Pegelwandler, Flash optional, Kabel-3V3 über 10 Ω, breitere 5-V- und Akku-Wege
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkZzubjLKyW9odUwvmxTog
</commit_message>
<xml_diff>
--- a/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
+++ b/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G55"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -502,7 +502,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>SPI-NAND 1 Gbit WSON-8 8x6</t>
+          <t>SPI-NAND 1 Gbit WSON-8 8x6 (optional)</t>
         </is>
       </c>
       <c r="F3" t="n">
@@ -510,7 +510,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Ersatz für ZD35Q1GC-IB (gleiches Gehäuse und Pinbelegung, von spi_nand_flash unterstützt)</t>
+          <t>Ersatz für ZD35Q1GC-IB (gleiches Gehäuse und Pinbelegung, von spi_nand_flash unterstützt); nur mit Flash bestücken, dazu C25 und R27</t>
         </is>
       </c>
     </row>
@@ -550,12 +550,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>74HCT125PW,118</t>
+          <t>MAX98357AETE+T</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nexperia</t>
+          <t>Analog Devices / Maxim</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -563,12 +563,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>U5</t>
+          <t>U6</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Puffer TSSOP-14</t>
+          <t>I2S-Verstärker TQFN-16</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -578,12 +578,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MAX98357AETE+T</t>
+          <t>USBLC6-2SC6</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Analog Devices / Maxim</t>
+          <t>STMicroelectronics</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -591,12 +591,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>U6</t>
+          <t>U12</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>I2S-Verstärker TQFN-16</t>
+          <t>USB-ESD SOT-23-6</t>
         </is>
       </c>
       <c r="F6" t="n">
@@ -606,35 +606,40 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>USBLC6-2SC6</t>
+          <t>DMN3404L-7</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>STMicroelectronics</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>U12</t>
+          <t>Q1,Q2</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>USB-ESD SOT-23-6</t>
+          <t>N-MOSFET 30 V SOT-23</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Ersatz für AO3400A (gleiche Pinbelegung)</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DMN3404L-7</t>
+          <t>2N7002-7-F</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -647,21 +652,16 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Q1,Q2</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>N-MOSFET 30 V SOT-23</t>
+          <t>N-MOSFET 60 V SOT-23 (WS2812-Pegelwandler)</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>Ersatz für AO3400A (gleiche Pinbelegung)</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -724,6 +724,11 @@
       <c r="F10" t="n">
         <v>1</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Ersatz für LBAT54CWT1G (kleiner Sperrstrom wichtig)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -761,7 +766,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CL32A107MPVNNNE</t>
+          <t>CL21A106KAYNNNE</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -770,26 +775,26 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>33</v>
+        <v>44</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C1,C7,C10</t>
+          <t>C2,C4,C18,C22</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MLCC 100 µF 10 V X5R 1210</t>
+          <t>MLCC 10 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CL21A106KAYNNNE</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -798,82 +803,82 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C2,C4,C18,C22</t>
+          <t>C28,C29</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 25 V X5R 0805</t>
+          <t>MLCC 10 µF 10 V X5R 0603</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C28,C29</t>
+          <t>C1,C7,C10,C19,C20,C30,C31,C32</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 10 V X5R 0603</t>
+          <t>MLCC 22 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GRM21BR61E226ME44L</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C19,C20,C30</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 25 V X5R 0805</t>
+          <t>MLCC 1 µF 50 V X5R 0603</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CL10A105KB8NNNC</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -882,16 +887,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MLCC 1 µF 50 V X5R 0603</t>
+          <t>MLCC 22 µF 6,3 V X5R 0603 (IP5306 BAT)</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -901,124 +906,134 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CL10A226MQ8NRNC</t>
+          <t>CC0603KRX7R9BB104</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>11</v>
+        <v>80</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C6,C8,C9,C17,C23,C25</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 6,3 V X5R 0603 (IP5306 BAT)</t>
+          <t>MLCC 100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>C25 nur mit Flash</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CC0603KRX7R9BB104</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C6,C8,C9,C17,C21,C23,C25</t>
+          <t>C26,C27</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 50 V X7R 0603</t>
+          <t>MLCC 100 nF 16 V X7R 0402</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>TAJA106K016RNJ</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Kyocera AVX</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C26,C27</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 16 V X7R 0402</t>
+          <t>Tantal 10 µF 16 V Case A</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TAJA106K016RNJ</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Kyocera AVX</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>11</v>
+        <v>70</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>R9,R10,R21,R24,R27</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tantal 10 µF 16 V Case A</t>
+          <t>10 kΩ 0603</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Polung beachten</t>
+          <t>R27 nur mit Flash</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>RC0603FR-071KL</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1027,26 +1042,26 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>R9,R10,R21,R24,R27</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>10 kΩ 0603</t>
+          <t>1 kΩ 0603</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-0710RL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1055,26 +1070,26 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>R6,R12</t>
+          <t>R36</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>100 kΩ 0603</t>
+          <t>10 Ω 0603 (3V3 J6)</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RC0603FR-071ML</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1087,12 +1102,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>R3,R4</t>
+          <t>R6,R12</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1 MΩ 0603</t>
+          <t>100 kΩ 0603</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1102,7 +1117,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RC0603FR-072RL</t>
+          <t>RC0603FR-071ML</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1111,26 +1126,26 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R3,R4</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2 Ω 0603</t>
+          <t>1 MΩ 0603</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RC0603FR-071RL</t>
+          <t>RC0603FR-072RL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1143,12 +1158,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1 Ω 0603</t>
+          <t>2 Ω 0603</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -1158,7 +1173,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RC0603FR-07100RL</t>
+          <t>RC0603FR-071RL</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1167,26 +1182,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R5,R11</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>100 Ω 0603</t>
+          <t>1 Ω 0603</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RC0603FR-07330RL</t>
+          <t>RC0603FR-07100RL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1195,26 +1210,26 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R5,R11</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>330 Ω 0603</t>
+          <t>100 Ω 0603</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RC0603FR-075K1L</t>
+          <t>RC0603FR-07330RL</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1223,26 +1238,26 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>R22,R23</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>5,1 kΩ 0603</t>
+          <t>330 Ω 0603</t>
         </is>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RC1206FR-0712RL</t>
+          <t>RC0603FR-075K1L</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1251,26 +1266,26 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R22,R23</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>12 Ω 1206</t>
+          <t>5,1 kΩ 0603</t>
         </is>
       </c>
       <c r="F29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RC0402FR-07100RL</t>
+          <t>RC1206FR-0722RL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1279,26 +1294,26 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>R28,R30,R31,R32,R33,R34</t>
+          <t>R7,R8</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>100 Ω 0402</t>
+          <t>22 Ω 1206</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RC0402FR-071KL</t>
+          <t>RC0402FR-07100RL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1307,26 +1322,26 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R28,R30,R31,R32,R33,R34</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1 kΩ 0402</t>
+          <t>100 Ω 0402</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RC0402FR-0710KL</t>
+          <t>RC0402FR-071KL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1339,12 +1354,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>10 kΩ 0402</t>
+          <t>1 kΩ 0402</t>
         </is>
       </c>
       <c r="F32" t="n">
@@ -1354,7 +1369,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RC0402FR-074K7L</t>
+          <t>RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1363,44 +1378,44 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>R38,R40</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>4,7 kΩ 0402</t>
+          <t>10 kΩ 0402</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>B3U-1000P</t>
+          <t>RC0402FR-074K7L</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>SW3,SW4</t>
+          <t>R38,R40</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Taster RESET/BOOT</t>
+          <t>4,7 kΩ 0402</t>
         </is>
       </c>
       <c r="F34" t="n">
@@ -1410,25 +1425,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SM07B-SRSS-TB(LF)(SN)</t>
+          <t>RC0402FR-0710RL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>R35</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>JST-SH 7-polig liegend</t>
+          <t>10 Ω 0402 (3V3 Weste)</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1438,12 +1453,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN)</t>
+          <t>B3U-1000P</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1451,12 +1466,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>J4,J5</t>
+          <t>SW3,SW4</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>JST-SH 4-polig liegend</t>
+          <t>Taster RESET/BOOT</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1466,7 +1481,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SM03B-SRSS-TB(LF)(SN)</t>
+          <t>SM07B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1479,12 +1494,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>JST-SH 3-polig liegend</t>
+          <t>JST-SH 7-polig liegend</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1494,7 +1509,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SM02B-SRSS-TB(LF)(SN)</t>
+          <t>SM04B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1503,26 +1518,26 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>LED1,M1,SW1,SW2</t>
+          <t>J4,J5</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>JST-SH 2-polig liegend</t>
+          <t>JST-SH 4-polig liegend</t>
         </is>
       </c>
       <c r="F38" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>SM05B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1531,26 +1546,26 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>BT1,SP1</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>JST-PH 2-polig liegend</t>
+          <t>JST-SH 5-polig liegend (IR-LED + TSOP 6)</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>S3B-PH-SM4-TB(LF)(SN)</t>
+          <t>SM03B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1563,12 +1578,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>J8</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>JST-PH 3-polig liegend</t>
+          <t>JST-SH 3-polig liegend (Abzug + Nachladen)</t>
         </is>
       </c>
       <c r="F40" t="n">
@@ -1578,96 +1593,91 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TSOP34838</t>
+          <t>SM02B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>60</v>
+        <v>10</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>TSOP 1-6</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
+          <t>JST-SH 2-polig liegend</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-100R</t>
+          <t>S2B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>66</v>
+        <v>20</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Filter TSOP (R)</t>
+          <t>BT1,SP1</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>100 Ω THT am Sensor</t>
+          <t>JST-PH 2-polig liegend</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>EEU-FR1H4R7</t>
+          <t>S3B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Filter TSOP (C)</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Elko 4,7 µF 50 V radial am Sensor</t>
+          <t>JST-PH 3-polig liegend</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>6</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TSAL6100</t>
+          <t>TSOP34838</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1676,92 +1686,92 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>IR-LED</t>
+          <t>TSOP 1-6</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>IR-LED 940 nm 5 mm</t>
+          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>D2F-01</t>
+          <t>MFR-25FBF52-100R</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Abzugsschalter</t>
+          <t>Filter TSOP (R)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mikroschalter</t>
+          <t>100 Ω THT am Sensor</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PTS645SL50-2 LFS</t>
+          <t>EEU-FR1H4R7</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Nachladetaster</t>
+          <t>Filter TSOP (C)</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Taster 6x6x5 THT</t>
+          <t>Elko 4,7 µF 50 V radial am Sensor</t>
         </is>
       </c>
       <c r="F46" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Ersatz für K2-1102DP</t>
+          <t>Polung beachten</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>PEC11R-4215F-S0024</t>
+          <t>TSAL6100</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1769,60 +1779,55 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Drehgeber</t>
+          <t>IR-LED</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Drehgeber 24 Rasten mit Taster</t>
+          <t>IR-LED 940 nm 5 mm</t>
         </is>
       </c>
       <c r="F47" t="n">
         <v>1</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
-        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SHR-02V-S-B</t>
+          <t>D2F-01</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 2p</t>
+          <t>Abzugsschalter</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Gehäuse SH 2-polig</t>
+          <t>Mikroschalter</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SHR-03V-S-B</t>
+          <t>PTS645SL50-2 LFS</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1830,50 +1835,60 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 3p</t>
+          <t>Nachladetaster</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Gehäuse SH 3-polig</t>
+          <t>Taster 6x6x5 THT</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Ersatz für K2-1102DP</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SHR-04V-S-B</t>
+          <t>PEC11R-4215F-S0024</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 4p</t>
+          <t>Drehgeber</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Gehäuse SH 4-polig</t>
+          <t>Drehgeber 24 Rasten mit Taster</t>
         </is>
       </c>
       <c r="F50" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SHR-07V-S-B</t>
+          <t>SHR-02V-S-B</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1886,12 +1901,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 7p</t>
+          <t>Gegenstecker SH 2p</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Gehäuse SH 7-polig</t>
+          <t>Gehäuse SH 2-polig</t>
         </is>
       </c>
       <c r="F51" t="n">
@@ -1901,7 +1916,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>SHR-03V-S-B</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1910,26 +1925,26 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>286</v>
+        <v>10</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Kontakte SH</t>
+          <t>Gegenstecker SH 3p</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Crimpkontakt SH AWG 32-28</t>
+          <t>Gehäuse SH 3-polig</t>
         </is>
       </c>
       <c r="F52" t="n">
-        <v>26</v>
+        <v>1</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>PHR-2</t>
+          <t>SHR-04V-S-B</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1942,12 +1957,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 2p</t>
+          <t>Gegenstecker SH 4p</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Gehäuse PH 2-polig</t>
+          <t>Gehäuse SH 4-polig</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -1957,7 +1972,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PHR-3</t>
+          <t>SHR-05V-S-B</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1970,12 +1985,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 3p</t>
+          <t>Gegenstecker SH 5p</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Gehäuse PH 3-polig</t>
+          <t>Gehäuse SH 5-polig</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -1985,28 +2000,140 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
+          <t>SHR-07V-S-B</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Gegenstecker SH 7p</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Gehäuse SH 7-polig</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>SSH-003T-P0.2-H</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>275</v>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Kontakte SH</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Crimpkontakt SH AWG 32-28</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>PHR-2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>20</v>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Gegenstecker PH 2p</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Gehäuse PH 2-polig</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>PHR-3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>10</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Gegenstecker PH 3p</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Gehäuse PH 3-polig</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>SPH-002T-P0.5S</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>JST</t>
         </is>
       </c>
-      <c r="C55" t="n">
+      <c r="C59" t="n">
         <v>77</v>
       </c>
-      <c r="D55" t="inlineStr">
+      <c r="D59" t="inlineStr">
         <is>
           <t>Kontakte PH</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr">
+      <c r="E59" t="inlineStr">
         <is>
           <t>Crimpkontakt PH AWG 30-24</t>
         </is>
       </c>
-      <c r="F55" t="n">
+      <c r="F59" t="n">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Platine: Lastschalter TPS22810 hinter dem IP5306 (EN = IRQ), RESET in die Lasche, Dämpfung an der USB-Buchse
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KkZzubjLKyW9odUwvmxTog
</commit_message>
<xml_diff>
--- a/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
+++ b/kicad/waffe_elektronik/fertigung/mouser/mouser_bom_10_waffen.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -700,12 +700,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BAT54CW-7-F</t>
+          <t>TPS22810DBVR</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Diodes Inc.</t>
+          <t>Texas Instruments</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -713,32 +713,27 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>U16</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Doppel-Schottky gemeinsame Kathode SOT-323 (Ein/Aus-Taster)</t>
+          <t>Lastschalter 2 A SOT-23-6 (5 V hinter dem IP5306, EN = IRQ)</t>
         </is>
       </c>
       <c r="F10" t="n">
         <v>1</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>Ersatz für LBAT54CWT1G (kleiner Sperrstrom wichtig)</t>
-        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SRP5030T-1R0M</t>
+          <t>BAT54CW-7-F</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Diodes Inc.</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -746,12 +741,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Speicherdrossel 1 µH 5,7x5,2 (IP5306)</t>
+          <t>Doppel-Schottky gemeinsame Kathode SOT-323 (Ein/Aus-Taster)</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -759,42 +754,47 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Ersatz für Sunlord MWSA0503S-1R0MT (Pads überlappen)</t>
+          <t>Ersatz für LBAT54CWT1G (kleiner Sperrstrom wichtig)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CL21A106KAYNNNE</t>
+          <t>SRP5030T-1R0M</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>C2,C4,C18,C22</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 25 V X5R 0805</t>
+          <t>Speicherdrossel 1 µH 5,7x5,2 (IP5306)</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Ersatz für Sunlord MWSA0503S-1R0MT (Pads überlappen)</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CL10A106KP8NNNC</t>
+          <t>CL21A106KAYNNNE</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -803,82 +803,82 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>C28,C29</t>
+          <t>C2,C18,C22</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>MLCC 10 µF 10 V X5R 0603</t>
+          <t>MLCC 10 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GRM21BR61E226ME44L</t>
+          <t>CL10A106KP8NNNC</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Murata</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>88</v>
+        <v>44</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>C1,C7,C10,C19,C20,C30,C31,C32</t>
+          <t>C4,C28,C29,C30</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 25 V X5R 0805</t>
+          <t>MLCC 10 µF 10 V X5R 0603</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CL10A105KB8NNNC</t>
+          <t>GRM21BR61E226ME44L</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Murata</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>20</v>
+        <v>77</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>C16</t>
+          <t>C1,C7,C10,C19,C20,C31,C32</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>MLCC 1 µF 50 V X5R 0603</t>
+          <t>MLCC 22 µF 25 V X5R 0805</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CL10A226MQ8NRNC</t>
+          <t>CL10A105KB8NNNC</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -887,16 +887,16 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>C5</t>
+          <t>C16</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>MLCC 22 µF 6,3 V X5R 0603 (IP5306 BAT)</t>
+          <t>MLCC 1 µF 50 V X5R 0603</t>
         </is>
       </c>
       <c r="F16" t="n">
@@ -906,162 +906,157 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CC0603KRX7R9BB104</t>
+          <t>CL10A226MQ8NRNC</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>80</v>
+        <v>11</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>C6,C8,C9,C17,C23,C25</t>
+          <t>C5</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 50 V X7R 0603</t>
+          <t>MLCC 22 µF 6,3 V X5R 0603 (IP5306 BAT)</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>6</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>C25 nur mit Flash</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CL05B104KO5NNNC</t>
+          <t>CC0603KRX7R9BB104</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Samsung</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>C26,C27</t>
+          <t>C6,C8,C9,C17,C23,C25</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>MLCC 100 nF 16 V X7R 0402</t>
+          <t>MLCC 100 nF 50 V X7R 0603</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>C25 nur mit Flash</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TAJA106K016RNJ</t>
+          <t>CL05B104KO5NNNC</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Kyocera AVX</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>C3</t>
+          <t>C26,C27</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tantal 10 µF 16 V Case A</t>
+          <t>MLCC 100 nF 16 V X7R 0402</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RC0603FR-0710KL</t>
+          <t>CL05B103KB5NNNC</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Samsung</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>R9,R10,R21,R24,R27</t>
+          <t>C33</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>10 kΩ 0603</t>
+          <t>MLCC 10 nF 50 V X7R 0402 (Anstieg U16)</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>R27 nur mit Flash</t>
-        </is>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>RC0603FR-071KL</t>
+          <t>TAJA106K016RNJ</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>Kyocera AVX</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>R25</t>
+          <t>C3</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1 kΩ 0603</t>
+          <t>Tantal 10 µF 16 V Case A</t>
         </is>
       </c>
       <c r="F21" t="n">
         <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>RC0603FR-0710RL</t>
+          <t>RC0603FR-0710KL</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1070,26 +1065,31 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>R36</t>
+          <t>R9,R10,R21,R24,R27</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>10 Ω 0603 (3V3 J6)</t>
+          <t>10 kΩ 0603</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>5</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>R27 nur mit Flash</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RC0603FR-07100KL</t>
+          <t>RC0603FR-071KL</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1098,26 +1098,26 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>R6,R12</t>
+          <t>R25</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>100 kΩ 0603</t>
+          <t>1 kΩ 0603</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>RC0603FR-071ML</t>
+          <t>RC0603FR-0710RL</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1126,26 +1126,26 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>R3,R4</t>
+          <t>R36</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1 MΩ 0603</t>
+          <t>10 Ω 0603 (3V3 J6)</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>RC0603FR-072RL</t>
+          <t>RC0603FR-07100KL</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1154,26 +1154,26 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R6,R12,R42</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2 Ω 0603</t>
+          <t>100 kΩ 0603</t>
         </is>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RC0603FR-071RL</t>
+          <t>RC0603FR-071ML</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1182,26 +1182,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>R2</t>
+          <t>R3,R4</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>1 Ω 0603</t>
+          <t>1 MΩ 0603</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>RC0603FR-07100RL</t>
+          <t>RC0603FR-072RL</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1210,26 +1210,26 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>R5,R11</t>
+          <t>R1</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>100 Ω 0603</t>
+          <t>2 Ω 0603</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RC0603FR-07330RL</t>
+          <t>RC0603FR-071RL</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1242,12 +1242,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>R15</t>
+          <t>R2</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>330 Ω 0603</t>
+          <t>1 Ω 0603</t>
         </is>
       </c>
       <c r="F28" t="n">
@@ -1257,7 +1257,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>RC0603FR-075K1L</t>
+          <t>RC0603FR-07100RL</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1270,12 +1270,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>R22,R23</t>
+          <t>R5,R11</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>5,1 kΩ 0603</t>
+          <t>100 Ω 0603</t>
         </is>
       </c>
       <c r="F29" t="n">
@@ -1285,7 +1285,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RC1206FR-0722RL</t>
+          <t>RC0603FR-07330RL</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1294,26 +1294,26 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>R7,R8</t>
+          <t>R15</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>22 Ω 1206</t>
+          <t>330 Ω 0603</t>
         </is>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RC0402FR-07100RL</t>
+          <t>RC0603FR-075K1L</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1322,26 +1322,26 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>80</v>
+        <v>30</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>R28,R30,R31,R32,R33,R34</t>
+          <t>R22,R23</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>100 Ω 0402</t>
+          <t>5,1 kΩ 0603</t>
         </is>
       </c>
       <c r="F31" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>RC0402FR-071KL</t>
+          <t>RC1206FR-0722RL</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1350,26 +1350,26 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R7,R8</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1 kΩ 0402</t>
+          <t>22 Ω 1206</t>
         </is>
       </c>
       <c r="F32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>RC0402FR-0710KL</t>
+          <t>RC0402FR-07100RL</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1378,26 +1378,26 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>R37</t>
+          <t>R28,R30,R31,R32,R33,R34</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>10 kΩ 0402</t>
+          <t>100 Ω 0402</t>
         </is>
       </c>
       <c r="F33" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RC0402FR-074K7L</t>
+          <t>RC0402FR-071KL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1406,26 +1406,26 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>R38,R40</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>4,7 kΩ 0402</t>
+          <t>1 kΩ 0402</t>
         </is>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>RC0402FR-0710RL</t>
+          <t>RC0402FR-0710KL</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1438,12 +1438,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>R35</t>
+          <t>R37</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>10 Ω 0402 (3V3 Weste)</t>
+          <t>10 kΩ 0402</t>
         </is>
       </c>
       <c r="F35" t="n">
@@ -1453,25 +1453,25 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>B3U-1000P</t>
+          <t>RC0402FR-074K7L</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>SW3,SW4</t>
+          <t>R38,R40</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Taster RESET/BOOT</t>
+          <t>4,7 kΩ 0402</t>
         </is>
       </c>
       <c r="F36" t="n">
@@ -1481,25 +1481,25 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SM07B-SRSS-TB(LF)(SN)</t>
+          <t>RC0402FR-0710RL</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>J2</t>
+          <t>R35</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>JST-SH 7-polig liegend</t>
+          <t>10 Ω 0402 (3V3 Weste)</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -1509,12 +1509,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SM04B-SRSS-TB(LF)(SN)</t>
+          <t>B3U-1000P</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1522,12 +1522,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>J4,J5</t>
+          <t>SW3,SW4</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>JST-SH 4-polig liegend</t>
+          <t>Taster RESET/BOOT</t>
         </is>
       </c>
       <c r="F38" t="n">
@@ -1537,7 +1537,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SM05B-SRSS-TB(LF)(SN)</t>
+          <t>SM07B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1550,12 +1550,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>J6</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>JST-SH 5-polig liegend (IR-LED + TSOP 6)</t>
+          <t>JST-SH 7-polig liegend</t>
         </is>
       </c>
       <c r="F39" t="n">
@@ -1565,7 +1565,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SM03B-SRSS-TB(LF)(SN)</t>
+          <t>SM04B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1574,26 +1574,26 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>J8</t>
+          <t>J4,J5</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>JST-SH 3-polig liegend (Abzug + Nachladen)</t>
+          <t>JST-SH 4-polig liegend</t>
         </is>
       </c>
       <c r="F40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SM02B-SRSS-TB(LF)(SN)</t>
+          <t>SM05B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1606,12 +1606,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>M1</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>JST-SH 2-polig liegend</t>
+          <t>JST-SH 5-polig liegend (IR-LED + TSOP 6)</t>
         </is>
       </c>
       <c r="F41" t="n">
@@ -1621,7 +1621,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>S2B-PH-SM4-TB(LF)(SN)</t>
+          <t>SM03B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1630,26 +1630,26 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>BT1,SP1</t>
+          <t>J8</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>JST-PH 2-polig liegend</t>
+          <t>JST-SH 3-polig liegend (Abzug + Nachladen)</t>
         </is>
       </c>
       <c r="F42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>S3B-PH-SM4-TB(LF)(SN)</t>
+          <t>SM02B-SRSS-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1662,12 +1662,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>M1</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>JST-PH 3-polig liegend</t>
+          <t>JST-SH 2-polig liegend</t>
         </is>
       </c>
       <c r="F43" t="n">
@@ -1677,157 +1677,157 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TSOP34838</t>
+          <t>S2B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>TSOP 1-6</t>
+          <t>BT1,SP1</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
+          <t>JST-PH 2-polig liegend</t>
         </is>
       </c>
       <c r="F44" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>MFR-25FBF52-100R</t>
+          <t>S3B-PH-SM4-TB(LF)(SN)</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Yageo</t>
+          <t>JST</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Filter TSOP (R)</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>100 Ω THT am Sensor</t>
+          <t>JST-PH 3-polig liegend</t>
         </is>
       </c>
       <c r="F45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>EEU-FR1H4R7</t>
+          <t>TSOP34838</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Panasonic</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Filter TSOP (C)</t>
+          <t>TSOP 1-6</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Elko 4,7 µF 50 V radial am Sensor</t>
+          <t>IR-Empfänger 38 kHz (5 Weste + 1 Waffe)</t>
         </is>
       </c>
       <c r="F46" t="n">
         <v>6</v>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>Polung beachten</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TSAL6100</t>
+          <t>MFR-25FBF52-100R</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Vishay</t>
+          <t>Yageo</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>IR-LED</t>
+          <t>Filter TSOP (R)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>IR-LED 940 nm 5 mm</t>
+          <t>100 Ω THT am Sensor</t>
         </is>
       </c>
       <c r="F47" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>D2F-01</t>
+          <t>EEU-FR1H4R7</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Omron</t>
+          <t>Panasonic</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>10</v>
+        <v>66</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Abzugsschalter</t>
+          <t>Filter TSOP (C)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Mikroschalter</t>
+          <t>Elko 4,7 µF 50 V radial am Sensor</t>
         </is>
       </c>
       <c r="F48" t="n">
-        <v>1</v>
+        <v>6</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Polung beachten</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>PTS645SL50-2 LFS</t>
+          <t>TSAL6100</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>C&amp;K</t>
+          <t>Vishay</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1835,32 +1835,27 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Nachladetaster</t>
+          <t>IR-LED</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Taster 6x6x5 THT</t>
+          <t>IR-LED 940 nm 5 mm</t>
         </is>
       </c>
       <c r="F49" t="n">
         <v>1</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Ersatz für K2-1102DP</t>
-        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PEC11R-4215F-S0024</t>
+          <t>D2F-01</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Bourns</t>
+          <t>Omron</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1868,32 +1863,27 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Drehgeber</t>
+          <t>Abzugsschalter</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Drehgeber 24 Rasten mit Taster</t>
+          <t>Mikroschalter</t>
         </is>
       </c>
       <c r="F50" t="n">
         <v>1</v>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
-        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SHR-02V-S-B</t>
+          <t>PTS645SL50-2 LFS</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>C&amp;K</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1901,27 +1891,32 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 2p</t>
+          <t>Nachladetaster</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Gehäuse SH 2-polig</t>
+          <t>Taster 6x6x5 THT</t>
         </is>
       </c>
       <c r="F51" t="n">
         <v>1</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Ersatz für K2-1102DP</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SHR-03V-S-B</t>
+          <t>PEC11R-4215F-S0024</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>JST</t>
+          <t>Bourns</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1929,22 +1924,27 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 3p</t>
+          <t>Drehgeber</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Gehäuse SH 3-polig</t>
+          <t>Drehgeber 24 Rasten mit Taster</t>
         </is>
       </c>
       <c r="F52" t="n">
         <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Ersatz für EC11, Wellenlänge im Griff prüfen</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SHR-04V-S-B</t>
+          <t>SHR-02V-S-B</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1953,26 +1953,26 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 4p</t>
+          <t>Gegenstecker SH 2p</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Gehäuse SH 4-polig</t>
+          <t>Gehäuse SH 2-polig</t>
         </is>
       </c>
       <c r="F53" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SHR-05V-S-B</t>
+          <t>SHR-03V-S-B</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1985,12 +1985,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 5p</t>
+          <t>Gegenstecker SH 3p</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Gehäuse SH 5-polig</t>
+          <t>Gehäuse SH 3-polig</t>
         </is>
       </c>
       <c r="F54" t="n">
@@ -2000,7 +2000,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SHR-07V-S-B</t>
+          <t>SHR-04V-S-B</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2009,26 +2009,26 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Gegenstecker SH 7p</t>
+          <t>Gegenstecker SH 4p</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Gehäuse SH 7-polig</t>
+          <t>Gehäuse SH 4-polig</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SSH-003T-P0.2-H</t>
+          <t>SHR-05V-S-B</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2037,26 +2037,26 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>275</v>
+        <v>10</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Kontakte SH</t>
+          <t>Gegenstecker SH 5p</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Crimpkontakt SH AWG 32-28</t>
+          <t>Gehäuse SH 5-polig</t>
         </is>
       </c>
       <c r="F56" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PHR-2</t>
+          <t>SHR-07V-S-B</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2065,26 +2065,26 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 2p</t>
+          <t>Gegenstecker SH 7p</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Gehäuse PH 2-polig</t>
+          <t>Gehäuse SH 7-polig</t>
         </is>
       </c>
       <c r="F57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>PHR-3</t>
+          <t>SSH-003T-P0.2-H</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2093,47 +2093,103 @@
         </is>
       </c>
       <c r="C58" t="n">
-        <v>10</v>
+        <v>275</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Gegenstecker PH 3p</t>
+          <t>Kontakte SH</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Gehäuse PH 3-polig</t>
+          <t>Crimpkontakt SH AWG 32-28</t>
         </is>
       </c>
       <c r="F58" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
+          <t>PHR-2</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>20</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Gegenstecker PH 2p</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Gehäuse PH 2-polig</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>PHR-3</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>JST</t>
+        </is>
+      </c>
+      <c r="C60" t="n">
+        <v>10</v>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Gegenstecker PH 3p</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Gehäuse PH 3-polig</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>SPH-002T-P0.5S</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr">
+      <c r="B61" t="inlineStr">
         <is>
           <t>JST</t>
         </is>
       </c>
-      <c r="C59" t="n">
+      <c r="C61" t="n">
         <v>77</v>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D61" t="inlineStr">
         <is>
           <t>Kontakte PH</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E61" t="inlineStr">
         <is>
           <t>Crimpkontakt PH AWG 30-24</t>
         </is>
       </c>
-      <c r="F59" t="n">
+      <c r="F61" t="n">
         <v>7</v>
       </c>
     </row>

</xml_diff>